<commit_message>
v3: finalize revision package
</commit_message>
<xml_diff>
--- a/results/03_coord_baseline/Fig03_Uranian_Wing_Source.xlsx
+++ b/results/03_coord_baseline/Fig03_Uranian_Wing_Source.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,102 +420,102 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Bin_Index</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>X_Axis</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Sat_701_Mean_SSN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Sat_702_Mean_SSN</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Sat_703_Mean_SSN</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Sat_704_Mean_SSN</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Sat_705_Mean_SSN</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Sat_706_Mean_SSN</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Sat_707_Mean_SSN</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Sat_708_Mean_SSN</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Sat_709_Mean_SSN</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Sat_710_Mean_SSN</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Sat_711_Mean_SSN</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Sat_712_Mean_SSN</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Sat_713_Mean_SSN</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Sat_714_Mean_SSN</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Sat_715_Mean_SSN</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Sat_725_Mean_SSN</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Sat_726_Mean_SSN</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Sat_727_Mean_SSN</t>
         </is>
@@ -12944,26 +12932,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Satellite_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Chi2_Stat</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>Chi2_P</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Cyclic_P</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Shuffle_P</t>
         </is>
@@ -12974,12 +12967,15 @@
         <v>701</v>
       </c>
       <c r="B2" t="n">
+        <v>6370.186448561903</v>
+      </c>
+      <c r="C2" t="n">
         <v>0</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>0.2791720827917208</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -12988,12 +12984,15 @@
         <v>702</v>
       </c>
       <c r="B3" t="n">
+        <v>6461.554771687727</v>
+      </c>
+      <c r="C3" t="n">
         <v>0</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>0.3312668733126687</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13002,12 +13001,15 @@
         <v>703</v>
       </c>
       <c r="B4" t="n">
+        <v>6555.782231180711</v>
+      </c>
+      <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>0.2750724927507249</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13016,12 +13018,15 @@
         <v>704</v>
       </c>
       <c r="B5" t="n">
+        <v>6313.80378323901</v>
+      </c>
+      <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>0.3086691330866913</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13030,12 +13035,15 @@
         <v>705</v>
       </c>
       <c r="B6" t="n">
+        <v>5674.479804636017</v>
+      </c>
+      <c r="C6" t="n">
         <v>0</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>0.5892410758924107</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13044,12 +13052,15 @@
         <v>706</v>
       </c>
       <c r="B7" t="n">
+        <v>2208.751561749159</v>
+      </c>
+      <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>0.116988301169883</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13058,12 +13069,15 @@
         <v>707</v>
       </c>
       <c r="B8" t="n">
+        <v>2404.450744834215</v>
+      </c>
+      <c r="C8" t="n">
         <v>0</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>0.101989801019898</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13072,12 +13086,15 @@
         <v>708</v>
       </c>
       <c r="B9" t="n">
+        <v>2267.401249399328</v>
+      </c>
+      <c r="C9" t="n">
         <v>0</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>0.06809319068093191</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13086,12 +13103,15 @@
         <v>709</v>
       </c>
       <c r="B10" t="n">
+        <v>2193.326285439693</v>
+      </c>
+      <c r="C10" t="n">
         <v>0</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>0.0725927407259274</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13100,12 +13120,15 @@
         <v>710</v>
       </c>
       <c r="B11" t="n">
+        <v>2456.060547813551</v>
+      </c>
+      <c r="C11" t="n">
         <v>0</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>0.07479252074792521</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13114,12 +13137,15 @@
         <v>711</v>
       </c>
       <c r="B12" t="n">
+        <v>2199.477174435367</v>
+      </c>
+      <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="n">
         <v>0.07989201079892011</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13128,12 +13154,15 @@
         <v>712</v>
       </c>
       <c r="B13" t="n">
+        <v>2291.764536280634</v>
+      </c>
+      <c r="C13" t="n">
         <v>0</v>
       </c>
-      <c r="C13" t="n">
+      <c r="D13" t="n">
         <v>0.09559044095590441</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13142,12 +13171,15 @@
         <v>713</v>
       </c>
       <c r="B14" t="n">
+        <v>2271.077366650649</v>
+      </c>
+      <c r="C14" t="n">
         <v>0</v>
       </c>
-      <c r="C14" t="n">
+      <c r="D14" t="n">
         <v>0.1076892310768923</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13156,12 +13188,15 @@
         <v>714</v>
       </c>
       <c r="B15" t="n">
+        <v>2388.304661220567</v>
+      </c>
+      <c r="C15" t="n">
         <v>0</v>
       </c>
-      <c r="C15" t="n">
+      <c r="D15" t="n">
         <v>0.09299070092990701</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13170,12 +13205,15 @@
         <v>715</v>
       </c>
       <c r="B16" t="n">
+        <v>2309.568476693898</v>
+      </c>
+      <c r="C16" t="n">
         <v>0</v>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="n">
         <v>0.1016898310168983</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13184,12 +13222,15 @@
         <v>725</v>
       </c>
       <c r="B17" t="n">
+        <v>2230.784238346949</v>
+      </c>
+      <c r="C17" t="n">
         <v>0</v>
       </c>
-      <c r="C17" t="n">
+      <c r="D17" t="n">
         <v>0.0861913808619138</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13198,12 +13239,15 @@
         <v>726</v>
       </c>
       <c r="B18" t="n">
+        <v>2548.732340221048</v>
+      </c>
+      <c r="C18" t="n">
         <v>0</v>
       </c>
-      <c r="C18" t="n">
+      <c r="D18" t="n">
         <v>0.0821917808219178</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13212,12 +13256,15 @@
         <v>727</v>
       </c>
       <c r="B19" t="n">
+        <v>2238.064392119174</v>
+      </c>
+      <c r="C19" t="n">
         <v>0</v>
       </c>
-      <c r="C19" t="n">
+      <c r="D19" t="n">
         <v>0.1590840915908409</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>9.999000099990002e-05</v>
       </c>
     </row>
@@ -13236,22 +13283,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>X_Axis</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Y_Combined</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Y_Inclination</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Y_Distance</t>
         </is>
@@ -13276,13 +13323,13 @@
         <v>-98.5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.5701292827038069</v>
+        <v>0.5701292827038071</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5533316101628996</v>
+        <v>0.5533316101628994</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8438845951917385</v>
+        <v>0.8438845951917384</v>
       </c>
     </row>
     <row r="4">
@@ -13293,7 +13340,7 @@
         <v>0.6589791116939901</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7645900931604129</v>
+        <v>0.7645900931604124</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -13304,13 +13351,13 @@
         <v>-96.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.830806726222212</v>
+        <v>0.8308067262222125</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8548773313478353</v>
+        <v>0.8548773313478354</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7346087745699452</v>
+        <v>0.7346087745699451</v>
       </c>
     </row>
     <row r="6">
@@ -13318,13 +13365,13 @@
         <v>-95.5</v>
       </c>
       <c r="B6" t="n">
-        <v>0.8788090083020381</v>
+        <v>0.8788090083020387</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9268316030667308</v>
+        <v>0.9268316030667305</v>
       </c>
       <c r="D6" t="n">
-        <v>0.640454327416757</v>
+        <v>0.6404543274167573</v>
       </c>
     </row>
     <row r="7">
@@ -13335,10 +13382,10 @@
         <v>0.8580910676842974</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8784181899133735</v>
+        <v>0.8784181899133733</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8327479931898826</v>
+        <v>0.832747993189883</v>
       </c>
     </row>
     <row r="8">
@@ -13346,13 +13393,13 @@
         <v>-93.5</v>
       </c>
       <c r="B8" t="n">
-        <v>0.9166586588809894</v>
+        <v>0.9166586588809902</v>
       </c>
       <c r="C8" t="n">
-        <v>0.8720846784569759</v>
+        <v>0.8720846784569756</v>
       </c>
       <c r="D8" t="n">
-        <v>0.816583536027413</v>
+        <v>0.8165835360274134</v>
       </c>
     </row>
     <row r="9">
@@ -13363,10 +13410,10 @@
         <v>0.8857752764382696</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9436124218256501</v>
+        <v>0.9436124218256494</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5170396654691453</v>
+        <v>0.517039665469145</v>
       </c>
     </row>
     <row r="10">
@@ -13374,13 +13421,13 @@
         <v>-91.5</v>
       </c>
       <c r="B10" t="n">
-        <v>0.9181860521551287</v>
+        <v>0.9181860521551291</v>
       </c>
       <c r="C10" t="n">
-        <v>0.9948473801037144</v>
+        <v>0.9948473801037139</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5541061527117704</v>
+        <v>0.5541061527117702</v>
       </c>
     </row>
     <row r="11">
@@ -13391,10 +13438,10 @@
         <v>0.9099481169834489</v>
       </c>
       <c r="C11" t="n">
-        <v>0.9701009922984414</v>
+        <v>0.970100992298441</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3446638354971175</v>
+        <v>0.3446638354971177</v>
       </c>
     </row>
     <row r="12">
@@ -13402,13 +13449,13 @@
         <v>-89.5</v>
       </c>
       <c r="B12" t="n">
-        <v>0.920034786848233</v>
+        <v>0.9200347868482333</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9576065329048673</v>
+        <v>0.9576065329048666</v>
       </c>
       <c r="D12" t="n">
-        <v>0.4103572060618615</v>
+        <v>0.4103572060618613</v>
       </c>
     </row>
     <row r="13">
@@ -13419,10 +13466,10 @@
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>0.9826620006446274</v>
+        <v>0.9826620006446267</v>
       </c>
       <c r="D13" t="n">
-        <v>0.4339215502290429</v>
+        <v>0.4339215502290431</v>
       </c>
     </row>
     <row r="14">
@@ -13430,13 +13477,13 @@
         <v>-87.5</v>
       </c>
       <c r="B14" t="n">
-        <v>0.9526932718290473</v>
+        <v>0.9526932718290475</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>0.4473415281371259</v>
+        <v>0.4473415281371261</v>
       </c>
     </row>
     <row r="15">
@@ -13444,13 +13491,13 @@
         <v>-86.5</v>
       </c>
       <c r="B15" t="n">
-        <v>0.9574561212793653</v>
+        <v>0.9574561212793656</v>
       </c>
       <c r="C15" t="n">
-        <v>0.9936465196613629</v>
+        <v>0.9936465196613622</v>
       </c>
       <c r="D15" t="n">
-        <v>0.4562406525897308</v>
+        <v>0.4562406525897311</v>
       </c>
     </row>
     <row r="16">
@@ -13458,13 +13505,13 @@
         <v>-85.5</v>
       </c>
       <c r="B16" t="n">
-        <v>0.9396782260874059</v>
+        <v>0.9396782260874063</v>
       </c>
       <c r="C16" t="n">
         <v>0.9958274071033653</v>
       </c>
       <c r="D16" t="n">
-        <v>0.4626397873271937</v>
+        <v>0.4626397873271935</v>
       </c>
     </row>
     <row r="17">
@@ -13472,13 +13519,13 @@
         <v>-84.5</v>
       </c>
       <c r="B17" t="n">
-        <v>0.9348241708469139</v>
+        <v>0.9348241708469145</v>
       </c>
       <c r="C17" t="n">
-        <v>0.9996418421698857</v>
+        <v>0.9996418421698854</v>
       </c>
       <c r="D17" t="n">
-        <v>0.4674861062426789</v>
+        <v>0.4674861062426786</v>
       </c>
     </row>
     <row r="18">
@@ -13486,13 +13533,13 @@
         <v>-83.5</v>
       </c>
       <c r="B18" t="n">
-        <v>0.9504237461131312</v>
+        <v>0.950423746113132</v>
       </c>
       <c r="C18" t="n">
-        <v>0.9022084139331087</v>
+        <v>0.9022084139331085</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4712932888281461</v>
+        <v>0.4712932888281459</v>
       </c>
     </row>
     <row r="19">
@@ -13500,13 +13547,13 @@
         <v>-82.5</v>
       </c>
       <c r="B19" t="n">
-        <v>0.9422191298223839</v>
+        <v>0.9422191298223848</v>
       </c>
       <c r="C19" t="n">
-        <v>0.936050289253903</v>
+        <v>0.9360502892539027</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4743674845947118</v>
+        <v>0.4743674845947116</v>
       </c>
     </row>
     <row r="20">
@@ -13514,13 +13561,13 @@
         <v>-81.5</v>
       </c>
       <c r="B20" t="n">
-        <v>0.949005915299686</v>
+        <v>0.9490059152996863</v>
       </c>
       <c r="C20" t="n">
-        <v>0.9203255877950701</v>
+        <v>0.9203255877950698</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4769037854021088</v>
+        <v>0.4769037854021086</v>
       </c>
     </row>
     <row r="21">
@@ -13528,13 +13575,13 @@
         <v>-80.5</v>
       </c>
       <c r="B21" t="n">
-        <v>0.9073459952330268</v>
+        <v>0.9073459952330274</v>
       </c>
       <c r="C21" t="n">
-        <v>0.8922182310421599</v>
+        <v>0.8922182310421597</v>
       </c>
       <c r="D21" t="n">
-        <v>0.4790329350508588</v>
+        <v>0.4790329350508589</v>
       </c>
     </row>
     <row r="22">
@@ -13542,13 +13589,13 @@
         <v>-79.5</v>
       </c>
       <c r="B22" t="n">
-        <v>0.8590822225198615</v>
+        <v>0.859082222519862</v>
       </c>
       <c r="C22" t="n">
         <v>0.8686954244354625</v>
       </c>
       <c r="D22" t="n">
-        <v>0.4808460853500087</v>
+        <v>0.4808460853500089</v>
       </c>
     </row>
     <row r="23">
@@ -13556,13 +13603,13 @@
         <v>-78.5</v>
       </c>
       <c r="B23" t="n">
-        <v>0.8588143440805717</v>
+        <v>0.8588143440805713</v>
       </c>
       <c r="C23" t="n">
-        <v>0.8577225764872749</v>
+        <v>0.857722576487274</v>
       </c>
       <c r="D23" t="n">
-        <v>0.4824088493430208</v>
+        <v>0.482408849343021</v>
       </c>
     </row>
     <row r="24">
@@ -13573,10 +13620,10 @@
         <v>0.8427787165576837</v>
       </c>
       <c r="C24" t="n">
-        <v>0.8315160483471457</v>
+        <v>0.8315160483471453</v>
       </c>
       <c r="D24" t="n">
-        <v>0.4837697231935115</v>
+        <v>0.4837697231935117</v>
       </c>
     </row>
     <row r="25">
@@ -13584,13 +13631,13 @@
         <v>-76.5</v>
       </c>
       <c r="B25" t="n">
-        <v>0.8234536853907762</v>
+        <v>0.8234536853907765</v>
       </c>
       <c r="C25" t="n">
-        <v>0.8038133418703667</v>
+        <v>0.8038133418703661</v>
       </c>
       <c r="D25" t="n">
-        <v>0.4849653605638656</v>
+        <v>0.4849653605638654</v>
       </c>
     </row>
     <row r="26">
@@ -13598,13 +13645,13 @@
         <v>-75.5</v>
       </c>
       <c r="B26" t="n">
-        <v>0.8226512579916015</v>
+        <v>0.8226512579916018</v>
       </c>
       <c r="C26" t="n">
-        <v>0.7559103261366089</v>
+        <v>0.755910326136608</v>
       </c>
       <c r="D26" t="n">
-        <v>0.486023998960846</v>
+        <v>0.4860239989608462</v>
       </c>
     </row>
     <row r="27">
@@ -13612,13 +13659,13 @@
         <v>-74.5</v>
       </c>
       <c r="B27" t="n">
-        <v>0.7944189533381556</v>
+        <v>0.7944189533381555</v>
       </c>
       <c r="C27" t="n">
-        <v>0.7574846670879898</v>
+        <v>0.7574846670879899</v>
       </c>
       <c r="D27" t="n">
-        <v>0.4869677555819383</v>
+        <v>0.4869677555819381</v>
       </c>
     </row>
     <row r="28">
@@ -13626,13 +13673,13 @@
         <v>-73.5</v>
       </c>
       <c r="B28" t="n">
-        <v>0.7614903717084363</v>
+        <v>0.7614903717084365</v>
       </c>
       <c r="C28" t="n">
-        <v>0.7317342294921181</v>
+        <v>0.7317342294921179</v>
       </c>
       <c r="D28" t="n">
-        <v>0.4878142071232827</v>
+        <v>0.4878142071232824</v>
       </c>
     </row>
     <row r="29">
@@ -13640,13 +13687,13 @@
         <v>-72.5</v>
       </c>
       <c r="B29" t="n">
-        <v>0.7525718692087209</v>
+        <v>0.7525718692087211</v>
       </c>
       <c r="C29" t="n">
-        <v>0.6846515295886507</v>
+        <v>0.6846515295886506</v>
       </c>
       <c r="D29" t="n">
-        <v>0.4885775022900861</v>
+        <v>0.4885775022900855</v>
       </c>
     </row>
     <row r="30">
@@ -13654,13 +13701,13 @@
         <v>-71.5</v>
       </c>
       <c r="B30" t="n">
-        <v>0.7551819610901543</v>
+        <v>0.7551819610901546</v>
       </c>
       <c r="C30" t="n">
-        <v>0.6651581063795067</v>
+        <v>0.6651581063795066</v>
       </c>
       <c r="D30" t="n">
-        <v>0.4892691612972991</v>
+        <v>0.4892691612972989</v>
       </c>
     </row>
     <row r="31">
@@ -13668,13 +13715,13 @@
         <v>-70.5</v>
       </c>
       <c r="B31" t="n">
-        <v>0.7359459575879775</v>
+        <v>0.7359459575879777</v>
       </c>
       <c r="C31" t="n">
-        <v>0.663419677775356</v>
+        <v>0.6634196777753558</v>
       </c>
       <c r="D31" t="n">
-        <v>0.4898986608521688</v>
+        <v>0.4898986608521677</v>
       </c>
     </row>
     <row r="32">
@@ -13682,13 +13729,13 @@
         <v>-69.5</v>
       </c>
       <c r="B32" t="n">
-        <v>0.7403937167767312</v>
+        <v>0.7403937167767317</v>
       </c>
       <c r="C32" t="n">
-        <v>0.6984860950493469</v>
+        <v>0.6984860950493468</v>
       </c>
       <c r="D32" t="n">
-        <v>0.4904738691034787</v>
+        <v>0.4904738691034785</v>
       </c>
     </row>
     <row r="33">
@@ -13699,10 +13746,10 @@
         <v>0.6968852396108124</v>
       </c>
       <c r="C33" t="n">
-        <v>0.6532069208884197</v>
+        <v>0.6532069208884193</v>
       </c>
       <c r="D33" t="n">
-        <v>0.4910013737367041</v>
+        <v>0.491001373736703</v>
       </c>
     </row>
     <row r="34">
@@ -13710,13 +13757,13 @@
         <v>-67.5</v>
       </c>
       <c r="B34" t="n">
-        <v>0.6854921487171532</v>
+        <v>0.6854921487171537</v>
       </c>
       <c r="C34" t="n">
-        <v>0.6282920299046594</v>
+        <v>0.6282920299046593</v>
       </c>
       <c r="D34" t="n">
-        <v>0.4914867327150998</v>
+        <v>0.4914867327150996</v>
       </c>
     </row>
     <row r="35">
@@ -13724,13 +13771,13 @@
         <v>-66.5</v>
       </c>
       <c r="B35" t="n">
-        <v>0.6704217975309409</v>
+        <v>0.6704217975309414</v>
       </c>
       <c r="C35" t="n">
-        <v>0.6100115711576957</v>
+        <v>0.6100115711576956</v>
       </c>
       <c r="D35" t="n">
-        <v>0.4919346681893128</v>
+        <v>0.4919346681893125</v>
       </c>
     </row>
     <row r="36">
@@ -13738,13 +13785,13 @@
         <v>-65.5</v>
       </c>
       <c r="B36" t="n">
-        <v>0.6343327075976388</v>
+        <v>0.6343327075976387</v>
       </c>
       <c r="C36" t="n">
-        <v>0.5956839979554051</v>
+        <v>0.5956839979554049</v>
       </c>
       <c r="D36" t="n">
-        <v>0.4923492180885909</v>
+        <v>0.4923492180885911</v>
       </c>
     </row>
     <row r="37">
@@ -13752,13 +13799,13 @@
         <v>-64.5</v>
       </c>
       <c r="B37" t="n">
-        <v>0.6515817250481675</v>
+        <v>0.6515817250481679</v>
       </c>
       <c r="C37" t="n">
-        <v>0.612716109480149</v>
+        <v>0.6127161094801492</v>
       </c>
       <c r="D37" t="n">
-        <v>0.4927338558112788</v>
+        <v>0.4927338558112785</v>
       </c>
     </row>
     <row r="38">
@@ -13766,13 +13813,13 @@
         <v>-63.5</v>
       </c>
       <c r="B38" t="n">
-        <v>0.6080531387907387</v>
+        <v>0.608053138790739</v>
       </c>
       <c r="C38" t="n">
-        <v>0.6023853488338297</v>
+        <v>0.6023853488338292</v>
       </c>
       <c r="D38" t="n">
-        <v>0.4930915855952366</v>
+        <v>0.4930915855952364</v>
       </c>
     </row>
     <row r="39">
@@ -13780,13 +13827,13 @@
         <v>-62.5</v>
       </c>
       <c r="B39" t="n">
-        <v>0.6133028294805949</v>
+        <v>0.6133028294805953</v>
       </c>
       <c r="C39" t="n">
-        <v>0.6030626920559258</v>
+        <v>0.6030626920559257</v>
       </c>
       <c r="D39" t="n">
-        <v>0.4934250191540233</v>
+        <v>0.4934250191540226</v>
       </c>
     </row>
     <row r="40">
@@ -13794,13 +13841,13 @@
         <v>-61.5</v>
       </c>
       <c r="B40" t="n">
-        <v>0.6282769128884991</v>
+        <v>0.6282769128884992</v>
       </c>
       <c r="C40" t="n">
-        <v>0.6205640652875102</v>
+        <v>0.62056406528751</v>
       </c>
       <c r="D40" t="n">
-        <v>0.493736437742581</v>
+        <v>0.4937364377425812</v>
       </c>
     </row>
     <row r="41">
@@ -13808,13 +13855,13 @@
         <v>-60.5</v>
       </c>
       <c r="B41" t="n">
-        <v>0.6079992034749827</v>
+        <v>0.6079992034749826</v>
       </c>
       <c r="C41" t="n">
-        <v>0.6152754383834582</v>
+        <v>0.615275438383458</v>
       </c>
       <c r="D41" t="n">
-        <v>0.4940278427895055</v>
+        <v>0.4940278427895053</v>
       </c>
     </row>
     <row r="42">
@@ -13822,13 +13869,13 @@
         <v>-59.5</v>
       </c>
       <c r="B42" t="n">
-        <v>0.5994710980975342</v>
+        <v>0.5994710980975344</v>
       </c>
       <c r="C42" t="n">
-        <v>0.6282379761625425</v>
+        <v>0.6282379761625431</v>
       </c>
       <c r="D42" t="n">
-        <v>0.4943009974829747</v>
+        <v>0.494300997482974</v>
       </c>
     </row>
     <row r="43">
@@ -13836,13 +13883,13 @@
         <v>-58.5</v>
       </c>
       <c r="B43" t="n">
-        <v>0.6099279444003927</v>
+        <v>0.6099279444003929</v>
       </c>
       <c r="C43" t="n">
-        <v>0.6414397726211378</v>
+        <v>0.641439772621138</v>
       </c>
       <c r="D43" t="n">
-        <v>0.4945574611436202</v>
+        <v>0.4945574611436195</v>
       </c>
     </row>
     <row r="44">
@@ -13850,13 +13897,13 @@
         <v>-57.5</v>
       </c>
       <c r="B44" t="n">
-        <v>0.6043557745641925</v>
+        <v>0.6043557745641932</v>
       </c>
       <c r="C44" t="n">
-        <v>0.6196484289744897</v>
+        <v>0.6196484289744902</v>
       </c>
       <c r="D44" t="n">
-        <v>0.4947986178044071</v>
+        <v>0.4947986178044065</v>
       </c>
     </row>
     <row r="45">
@@ -13864,13 +13911,13 @@
         <v>-56.5</v>
       </c>
       <c r="B45" t="n">
-        <v>0.6269512787918737</v>
+        <v>0.6269512787918736</v>
       </c>
       <c r="C45" t="n">
-        <v>0.6219176561838072</v>
+        <v>0.6219176561838073</v>
       </c>
       <c r="D45" t="n">
-        <v>0.4950257001064756</v>
+        <v>0.4950257001064754</v>
       </c>
     </row>
     <row r="46">
@@ -13878,13 +13925,13 @@
         <v>-55.5</v>
       </c>
       <c r="B46" t="n">
-        <v>0.626859395629082</v>
+        <v>0.6268593956290824</v>
       </c>
       <c r="C46" t="n">
-        <v>0.6140979057477214</v>
+        <v>0.6140979057477209</v>
       </c>
       <c r="D46" t="n">
-        <v>0.4952398093834697</v>
+        <v>0.4952398093834686</v>
       </c>
     </row>
     <row r="47">
@@ -13892,13 +13939,13 @@
         <v>-54.5</v>
       </c>
       <c r="B47" t="n">
-        <v>0.6145222782996753</v>
+        <v>0.6145222782996752</v>
       </c>
       <c r="C47" t="n">
-        <v>0.6955921174697973</v>
+        <v>0.6955921174697978</v>
       </c>
       <c r="D47" t="n">
-        <v>0.4954419326257448</v>
+        <v>0.4954419326257442</v>
       </c>
     </row>
     <row r="48">
@@ -13906,13 +13953,13 @@
         <v>-53.5</v>
       </c>
       <c r="B48" t="n">
-        <v>0.6075886268367905</v>
+        <v>0.6075886268367907</v>
       </c>
       <c r="C48" t="n">
-        <v>0.6417492754696281</v>
+        <v>0.6417492754696279</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4956329568760179</v>
+        <v>0.4956329568760177</v>
       </c>
     </row>
     <row r="49">
@@ -13920,13 +13967,13 @@
         <v>-52.5</v>
       </c>
       <c r="B49" t="n">
-        <v>0.6621240246579133</v>
+        <v>0.6621240246579135</v>
       </c>
       <c r="C49" t="n">
-        <v>0.6608141905780918</v>
+        <v>0.660814190578092</v>
       </c>
       <c r="D49" t="n">
-        <v>0.495813681499212</v>
+        <v>0.4958136814992118</v>
       </c>
     </row>
     <row r="50">
@@ -13934,13 +13981,13 @@
         <v>-51.5</v>
       </c>
       <c r="B50" t="n">
-        <v>0.6482710607618596</v>
+        <v>0.6482710607618598</v>
       </c>
       <c r="C50" t="n">
-        <v>0.6444745327159636</v>
+        <v>0.6444745327159631</v>
       </c>
       <c r="D50" t="n">
-        <v>0.4959848286840581</v>
+        <v>0.4959848286840583</v>
       </c>
     </row>
     <row r="51">
@@ -13948,13 +13995,13 @@
         <v>-50.5</v>
       </c>
       <c r="B51" t="n">
-        <v>0.629700875046741</v>
+        <v>0.6297008750467409</v>
       </c>
       <c r="C51" t="n">
-        <v>0.6784468564926708</v>
+        <v>0.6784468564926709</v>
       </c>
       <c r="D51" t="n">
-        <v>0.4961470524668356</v>
+        <v>0.4961470524668354</v>
       </c>
     </row>
     <row r="52">
@@ -13962,13 +14009,13 @@
         <v>-49.5</v>
       </c>
       <c r="B52" t="n">
-        <v>0.6296245049056135</v>
+        <v>0.6296245049056137</v>
       </c>
       <c r="C52" t="n">
-        <v>0.7021565699010888</v>
+        <v>0.7021565699010887</v>
       </c>
       <c r="D52" t="n">
-        <v>0.496300946514333</v>
+        <v>0.4963009465143333</v>
       </c>
     </row>
     <row r="53">
@@ -13976,13 +14023,13 @@
         <v>-48.5</v>
       </c>
       <c r="B53" t="n">
-        <v>0.6422987617800502</v>
+        <v>0.6422987617800497</v>
       </c>
       <c r="C53" t="n">
-        <v>0.6828565450664376</v>
+        <v>0.6828565450664378</v>
       </c>
       <c r="D53" t="n">
-        <v>0.496447050860586</v>
+        <v>0.4964470508605858</v>
       </c>
     </row>
     <row r="54">
@@ -13990,13 +14037,13 @@
         <v>-47.5</v>
       </c>
       <c r="B54" t="n">
-        <v>0.6560576920298822</v>
+        <v>0.6560576920298824</v>
       </c>
       <c r="C54" t="n">
-        <v>0.6759809314377453</v>
+        <v>0.6759809314377454</v>
       </c>
       <c r="D54" t="n">
-        <v>0.4965858577578205</v>
+        <v>0.4965858577578208</v>
       </c>
     </row>
     <row r="55">
@@ -14004,13 +14051,13 @@
         <v>-46.5</v>
       </c>
       <c r="B55" t="n">
-        <v>0.6523653457907461</v>
+        <v>0.6523653457907458</v>
       </c>
       <c r="C55" t="n">
-        <v>0.6938881629172772</v>
+        <v>0.693888162917277</v>
       </c>
       <c r="D55" t="n">
-        <v>0.4967178167744916</v>
+        <v>0.4967178167744914</v>
       </c>
     </row>
     <row r="56">
@@ -14018,13 +14065,13 @@
         <v>-45.5</v>
       </c>
       <c r="B56" t="n">
-        <v>0.65703046610319</v>
+        <v>0.6570304661031902</v>
       </c>
       <c r="C56" t="n">
-        <v>0.6891287255111701</v>
+        <v>0.68912872551117</v>
       </c>
       <c r="D56" t="n">
-        <v>0.4968433392509789</v>
+        <v>0.4968433392509787</v>
       </c>
     </row>
     <row r="57">
@@ -14032,13 +14079,13 @@
         <v>-44.5</v>
       </c>
       <c r="B57" t="n">
-        <v>0.6579346460701211</v>
+        <v>0.6579346460701213</v>
       </c>
       <c r="C57" t="n">
-        <v>0.6855482572812029</v>
+        <v>0.6855482572812028</v>
       </c>
       <c r="D57" t="n">
-        <v>0.4969628022053188</v>
+        <v>0.4969628022053186</v>
       </c>
     </row>
     <row r="58">
@@ -14046,13 +14093,13 @@
         <v>-43.5</v>
       </c>
       <c r="B58" t="n">
-        <v>0.6614806547034983</v>
+        <v>0.6614806547034987</v>
       </c>
       <c r="C58" t="n">
-        <v>0.7007304608014034</v>
+        <v>0.700730460801403</v>
       </c>
       <c r="D58" t="n">
-        <v>0.497076551766442</v>
+        <v>0.4970765517664418</v>
       </c>
     </row>
     <row r="59">
@@ -14060,13 +14107,13 @@
         <v>-42.5</v>
       </c>
       <c r="B59" t="n">
-        <v>0.6656779753720748</v>
+        <v>0.6656779753720753</v>
       </c>
       <c r="C59" t="n">
-        <v>0.7346912850045731</v>
+        <v>0.734691285004573</v>
       </c>
       <c r="D59" t="n">
-        <v>0.4971849062001671</v>
+        <v>0.4971849062001669</v>
       </c>
     </row>
     <row r="60">
@@ -14074,13 +14121,13 @@
         <v>-41.5</v>
       </c>
       <c r="B60" t="n">
-        <v>0.6756810914760258</v>
+        <v>0.675681091476026</v>
       </c>
       <c r="C60" t="n">
-        <v>0.7475540536762612</v>
+        <v>0.7475540536762606</v>
       </c>
       <c r="D60" t="n">
-        <v>0.4972881585830732</v>
+        <v>0.497288158583073</v>
       </c>
     </row>
     <row r="61">
@@ -14088,13 +14135,13 @@
         <v>-40.5</v>
       </c>
       <c r="B61" t="n">
-        <v>0.6926928773884129</v>
+        <v>0.6926928773884131</v>
       </c>
       <c r="C61" t="n">
-        <v>0.7754443003335992</v>
+        <v>0.775444300333599</v>
       </c>
       <c r="D61" t="n">
-        <v>0.4973865791710019</v>
+        <v>0.4973865791710017</v>
       </c>
     </row>
     <row r="62">
@@ -14102,13 +14149,13 @@
         <v>-39.5</v>
       </c>
       <c r="B62" t="n">
-        <v>0.720475589674085</v>
+        <v>0.7204755896740852</v>
       </c>
       <c r="C62" t="n">
-        <v>0.8117217715841862</v>
+        <v>0.811721771584186</v>
       </c>
       <c r="D62" t="n">
-        <v>0.4974804175019663</v>
+        <v>0.4974804175019656</v>
       </c>
     </row>
     <row r="63">
@@ -14116,13 +14163,13 @@
         <v>-38.5</v>
       </c>
       <c r="B63" t="n">
-        <v>0.7536978025320183</v>
+        <v>0.7536978025320188</v>
       </c>
       <c r="C63" t="n">
-        <v>0.7751001179241852</v>
+        <v>0.7751001179241843</v>
       </c>
       <c r="D63" t="n">
-        <v>0.4975699042674191</v>
+        <v>0.4975699042674197</v>
       </c>
     </row>
     <row r="64">
@@ -14130,13 +14177,13 @@
         <v>-37.5</v>
       </c>
       <c r="B64" t="n">
-        <v>0.7920464134216572</v>
+        <v>0.7920464134216577</v>
       </c>
       <c r="C64" t="n">
-        <v>0.7711934302937643</v>
+        <v>0.7711934302937647</v>
       </c>
       <c r="D64" t="n">
-        <v>0.4976552529809558</v>
+        <v>0.497655252980956</v>
       </c>
     </row>
     <row r="65">
@@ -14144,13 +14191,13 @@
         <v>-36.5</v>
       </c>
       <c r="B65" t="n">
-        <v>0.7524199679378973</v>
+        <v>0.7524199679378979</v>
       </c>
       <c r="C65" t="n">
-        <v>0.7747048381020563</v>
+        <v>0.7747048381020564</v>
       </c>
       <c r="D65" t="n">
-        <v>0.4977366614693945</v>
+        <v>0.4977366614693943</v>
       </c>
     </row>
     <row r="66">
@@ -14158,13 +14205,13 @@
         <v>-35.5</v>
       </c>
       <c r="B66" t="n">
-        <v>0.7475877850546789</v>
+        <v>0.7475877850546786</v>
       </c>
       <c r="C66" t="n">
-        <v>0.7930276421197473</v>
+        <v>0.7930276421197467</v>
       </c>
       <c r="D66" t="n">
-        <v>0.4978143132077587</v>
+        <v>0.497814313207758</v>
       </c>
     </row>
     <row r="67">
@@ -14172,13 +14219,13 @@
         <v>-34.5</v>
       </c>
       <c r="B67" t="n">
-        <v>0.7786175759937868</v>
+        <v>0.778617575993787</v>
       </c>
       <c r="C67" t="n">
-        <v>0.7944551418583022</v>
+        <v>0.7944551418583017</v>
       </c>
       <c r="D67" t="n">
-        <v>0.4978883785166947</v>
+        <v>0.497888378516694</v>
       </c>
     </row>
     <row r="68">
@@ -14186,13 +14233,13 @@
         <v>-33.5</v>
       </c>
       <c r="B68" t="n">
-        <v>0.7850969335610457</v>
+        <v>0.7850969335610462</v>
       </c>
       <c r="C68" t="n">
-        <v>0.7966176111302646</v>
+        <v>0.7966176111302644</v>
       </c>
       <c r="D68" t="n">
-        <v>0.4979590156384209</v>
+        <v>0.4979590156384207</v>
       </c>
     </row>
     <row r="69">
@@ -14200,13 +14247,13 @@
         <v>-32.5</v>
       </c>
       <c r="B69" t="n">
-        <v>0.7658216424068954</v>
+        <v>0.7658216424068957</v>
       </c>
       <c r="C69" t="n">
-        <v>0.762833644079726</v>
+        <v>0.7628336440797258</v>
       </c>
       <c r="D69" t="n">
-        <v>0.4980263717051334</v>
+        <v>0.4980263717051331</v>
       </c>
     </row>
     <row r="70">
@@ -14217,10 +14264,10 @@
         <v>0.7621490712918519</v>
       </c>
       <c r="C70" t="n">
-        <v>0.7743819592484078</v>
+        <v>0.7743819592484076</v>
       </c>
       <c r="D70" t="n">
-        <v>0.4980905836120113</v>
+        <v>0.4980905836120115</v>
       </c>
     </row>
     <row r="71">
@@ -14228,13 +14275,13 @@
         <v>-30.5</v>
       </c>
       <c r="B71" t="n">
-        <v>0.7510838934016182</v>
+        <v>0.7510838934016184</v>
       </c>
       <c r="C71" t="n">
-        <v>0.7801299757621555</v>
+        <v>0.7801299757621549</v>
       </c>
       <c r="D71" t="n">
-        <v>0.4981517788054157</v>
+        <v>0.4981517788054154</v>
       </c>
     </row>
     <row r="72">
@@ -14242,13 +14289,13 @@
         <v>-29.5</v>
       </c>
       <c r="B72" t="n">
-        <v>0.754333178138484</v>
+        <v>0.7543331781384839</v>
       </c>
       <c r="C72" t="n">
-        <v>0.7798271559346585</v>
+        <v>0.7798271559346582</v>
       </c>
       <c r="D72" t="n">
-        <v>0.498210075995503</v>
+        <v>0.4982100759955033</v>
       </c>
     </row>
     <row r="73">
@@ -14256,13 +14303,13 @@
         <v>-28.5</v>
       </c>
       <c r="B73" t="n">
-        <v>0.7848787755905255</v>
+        <v>0.784878775590526</v>
       </c>
       <c r="C73" t="n">
-        <v>0.7822384288115791</v>
+        <v>0.7822384288115796</v>
       </c>
       <c r="D73" t="n">
-        <v>0.4982655858013817</v>
+        <v>0.4982655858013811</v>
       </c>
     </row>
     <row r="74">
@@ -14273,10 +14320,10 @@
         <v>0.7738232236139158</v>
       </c>
       <c r="C74" t="n">
-        <v>0.7700672377093174</v>
+        <v>0.7700672377093175</v>
       </c>
       <c r="D74" t="n">
-        <v>0.4983184113358945</v>
+        <v>0.4983184113358947</v>
       </c>
     </row>
     <row r="75">
@@ -14284,13 +14331,13 @@
         <v>-26.5</v>
       </c>
       <c r="B75" t="n">
-        <v>0.7595058745635348</v>
+        <v>0.7595058745635345</v>
       </c>
       <c r="C75" t="n">
-        <v>0.7595896469084757</v>
+        <v>0.7595896469084759</v>
       </c>
       <c r="D75" t="n">
-        <v>0.4983686487363029</v>
+        <v>0.4983686487363018</v>
       </c>
     </row>
     <row r="76">
@@ -14298,13 +14345,13 @@
         <v>-25.5</v>
       </c>
       <c r="B76" t="n">
-        <v>0.7453626901331355</v>
+        <v>0.7453626901331359</v>
       </c>
       <c r="C76" t="n">
-        <v>0.7717598754606786</v>
+        <v>0.7717598754606784</v>
       </c>
       <c r="D76" t="n">
-        <v>0.4984163876463492</v>
+        <v>0.4984163876463485</v>
       </c>
     </row>
     <row r="77">
@@ -14312,13 +14359,13 @@
         <v>-24.5</v>
       </c>
       <c r="B77" t="n">
-        <v>0.7333517317115432</v>
+        <v>0.7333517317115434</v>
       </c>
       <c r="C77" t="n">
-        <v>0.7264060933968987</v>
+        <v>0.7264060933968978</v>
       </c>
       <c r="D77" t="n">
-        <v>0.4984617116545876</v>
+        <v>0.498461711654587</v>
       </c>
     </row>
     <row r="78">
@@ -14326,13 +14373,13 @@
         <v>-23.5</v>
       </c>
       <c r="B78" t="n">
-        <v>0.6942382422069006</v>
+        <v>0.6942382422069008</v>
       </c>
       <c r="C78" t="n">
-        <v>0.6979243713813409</v>
+        <v>0.6979243713813407</v>
       </c>
       <c r="D78" t="n">
-        <v>0.4985046986932534</v>
+        <v>0.4985046986932536</v>
       </c>
     </row>
     <row r="79">
@@ -14340,13 +14387,13 @@
         <v>-22.5</v>
       </c>
       <c r="B79" t="n">
-        <v>0.7003159604390922</v>
+        <v>0.7003159604390918</v>
       </c>
       <c r="C79" t="n">
-        <v>0.6999179633507362</v>
+        <v>0.6999179633507361</v>
       </c>
       <c r="D79" t="n">
-        <v>0.4985454214014907</v>
+        <v>0.4985454214014905</v>
       </c>
     </row>
     <row r="80">
@@ -14354,13 +14401,13 @@
         <v>-21.5</v>
       </c>
       <c r="B80" t="n">
-        <v>0.7097767783035674</v>
+        <v>0.7097767783035679</v>
       </c>
       <c r="C80" t="n">
-        <v>0.6805365234859008</v>
+        <v>0.680536523485901</v>
       </c>
       <c r="D80" t="n">
-        <v>0.4985839474562871</v>
+        <v>0.4985839474562869</v>
       </c>
     </row>
     <row r="81">
@@ -14368,13 +14415,13 @@
         <v>-20.5</v>
       </c>
       <c r="B81" t="n">
-        <v>0.6813932420874094</v>
+        <v>0.6813932420874093</v>
       </c>
       <c r="C81" t="n">
-        <v>0.6598358656296602</v>
+        <v>0.6598358656296595</v>
       </c>
       <c r="D81" t="n">
-        <v>0.4986203398741444</v>
+        <v>0.4986203398741442</v>
       </c>
     </row>
     <row r="82">
@@ -14382,13 +14429,13 @@
         <v>-19.5</v>
       </c>
       <c r="B82" t="n">
-        <v>0.6769639820830026</v>
+        <v>0.6769639820830036</v>
       </c>
       <c r="C82" t="n">
-        <v>0.6608455717034396</v>
+        <v>0.66084557170344</v>
       </c>
       <c r="D82" t="n">
-        <v>0.4986546572861053</v>
+        <v>0.4986546572861046</v>
       </c>
     </row>
     <row r="83">
@@ -14396,13 +14443,13 @@
         <v>-18.5</v>
       </c>
       <c r="B83" t="n">
-        <v>0.671066575295569</v>
+        <v>0.6710665752955695</v>
       </c>
       <c r="C83" t="n">
-        <v>0.6467881970659735</v>
+        <v>0.6467881970659737</v>
       </c>
       <c r="D83" t="n">
-        <v>0.4986869541885289</v>
+        <v>0.4986869541885287</v>
       </c>
     </row>
     <row r="84">
@@ -14410,13 +14457,13 @@
         <v>-17.5</v>
       </c>
       <c r="B84" t="n">
-        <v>0.6404980446626786</v>
+        <v>0.6404980446626785</v>
       </c>
       <c r="C84" t="n">
-        <v>0.6101167302671517</v>
+        <v>0.6101167302671512</v>
       </c>
       <c r="D84" t="n">
-        <v>0.4987172811717101</v>
+        <v>0.4987172811717099</v>
       </c>
     </row>
     <row r="85">
@@ -14424,13 +14471,13 @@
         <v>-16.5</v>
       </c>
       <c r="B85" t="n">
-        <v>0.6669176724807067</v>
+        <v>0.6669176724807072</v>
       </c>
       <c r="C85" t="n">
-        <v>0.6332829617875403</v>
+        <v>0.6332829617875398</v>
       </c>
       <c r="D85" t="n">
-        <v>0.4987456851282283</v>
+        <v>0.4987456851282294</v>
       </c>
     </row>
     <row r="86">
@@ -14438,13 +14485,13 @@
         <v>-15.5</v>
       </c>
       <c r="B86" t="n">
-        <v>0.6469516045484214</v>
+        <v>0.6469516045484219</v>
       </c>
       <c r="C86" t="n">
-        <v>0.6133578052689883</v>
+        <v>0.6133578052689885</v>
       </c>
       <c r="D86" t="n">
-        <v>0.4987722094426909</v>
+        <v>0.4987722094426906</v>
       </c>
     </row>
     <row r="87">
@@ -14452,13 +14499,13 @@
         <v>-14.5</v>
       </c>
       <c r="B87" t="n">
-        <v>0.6209617681089237</v>
+        <v>0.6209617681089239</v>
       </c>
       <c r="C87" t="n">
-        <v>0.5921305698265923</v>
+        <v>0.5921305698265928</v>
       </c>
       <c r="D87" t="n">
-        <v>0.4987968941643666</v>
+        <v>0.4987968941643673</v>
       </c>
     </row>
     <row r="88">
@@ -14466,13 +14513,13 @@
         <v>-13.5</v>
       </c>
       <c r="B88" t="n">
-        <v>0.6011421029666544</v>
+        <v>0.6011421029666546</v>
       </c>
       <c r="C88" t="n">
-        <v>0.5670821387773938</v>
+        <v>0.5670821387773937</v>
       </c>
       <c r="D88" t="n">
-        <v>0.4988197761640505</v>
+        <v>0.4988197761640507</v>
       </c>
     </row>
     <row r="89">
@@ -14480,13 +14527,13 @@
         <v>-12.5</v>
       </c>
       <c r="B89" t="n">
-        <v>0.5788870879431407</v>
+        <v>0.5788870879431408</v>
       </c>
       <c r="C89" t="n">
-        <v>0.5325837617871744</v>
+        <v>0.5325837617871743</v>
       </c>
       <c r="D89" t="n">
-        <v>0.4988408892763265</v>
+        <v>0.4988408892763267</v>
       </c>
     </row>
     <row r="90">
@@ -14494,13 +14541,13 @@
         <v>-11.5</v>
       </c>
       <c r="B90" t="n">
-        <v>0.539122105997347</v>
+        <v>0.5391221059973471</v>
       </c>
       <c r="C90" t="n">
-        <v>0.5230233532025188</v>
+        <v>0.523023353202519</v>
       </c>
       <c r="D90" t="n">
-        <v>0.4988602644283019</v>
+        <v>0.4988602644283012</v>
       </c>
     </row>
     <row r="91">
@@ -14508,13 +14555,13 @@
         <v>-10.5</v>
       </c>
       <c r="B91" t="n">
-        <v>0.5303544982557074</v>
+        <v>0.530354498255708</v>
       </c>
       <c r="C91" t="n">
-        <v>0.4725330359338211</v>
+        <v>0.472533035933821</v>
       </c>
       <c r="D91" t="n">
-        <v>0.4988779297557414</v>
+        <v>0.4988779297557407</v>
       </c>
     </row>
     <row r="92">
@@ -14522,13 +14569,13 @@
         <v>-9.5</v>
       </c>
       <c r="B92" t="n">
-        <v>0.4999181578253317</v>
+        <v>0.4999181578253318</v>
       </c>
       <c r="C92" t="n">
-        <v>0.4653872301930296</v>
+        <v>0.4653872301930295</v>
       </c>
       <c r="D92" t="n">
-        <v>0.4988939107074428</v>
+        <v>0.4988939107074422</v>
       </c>
     </row>
     <row r="93">
@@ -14536,13 +14583,13 @@
         <v>-8.5</v>
       </c>
       <c r="B93" t="n">
-        <v>0.4820740942211141</v>
+        <v>0.4820740942211145</v>
       </c>
       <c r="C93" t="n">
         <v>0.4269853796058833</v>
       </c>
       <c r="D93" t="n">
-        <v>0.498908230138588</v>
+        <v>0.4989082301385873</v>
       </c>
     </row>
     <row r="94">
@@ -14550,13 +14597,13 @@
         <v>-7.5</v>
       </c>
       <c r="B94" t="n">
-        <v>0.4389426994509298</v>
+        <v>0.43894269945093</v>
       </c>
       <c r="C94" t="n">
-        <v>0.38792404962975</v>
+        <v>0.3879240496297497</v>
       </c>
       <c r="D94" t="n">
-        <v>0.4989209083937158</v>
+        <v>0.4989209083937156</v>
       </c>
     </row>
     <row r="95">
@@ -14564,13 +14611,13 @@
         <v>-6.5</v>
       </c>
       <c r="B95" t="n">
-        <v>0.4041074485698596</v>
+        <v>0.40410744856986</v>
       </c>
       <c r="C95" t="n">
         <v>0.3682076421570132</v>
       </c>
       <c r="D95" t="n">
-        <v>0.498931963379897</v>
+        <v>0.4989319633798968</v>
       </c>
     </row>
     <row r="96">
@@ -14578,13 +14625,13 @@
         <v>-5.5</v>
       </c>
       <c r="B96" t="n">
-        <v>0.3877315662205335</v>
+        <v>0.3877315662205336</v>
       </c>
       <c r="C96" t="n">
         <v>0.3342570787069619</v>
       </c>
       <c r="D96" t="n">
-        <v>0.4989414106306054</v>
+        <v>0.4989414106306061</v>
       </c>
     </row>
     <row r="97">
@@ -14592,13 +14639,13 @@
         <v>-4.5</v>
       </c>
       <c r="B97" t="n">
-        <v>0.3352972603430681</v>
+        <v>0.3352972603430684</v>
       </c>
       <c r="C97" t="n">
-        <v>0.2840653476254301</v>
+        <v>0.2840653476254295</v>
       </c>
       <c r="D97" t="n">
-        <v>0.4989492633607075</v>
+        <v>0.4989492633607073</v>
       </c>
     </row>
     <row r="98">
@@ -14606,13 +14653,13 @@
         <v>-3.5</v>
       </c>
       <c r="B98" t="n">
-        <v>0.300112390596965</v>
+        <v>0.3001123905969652</v>
       </c>
       <c r="C98" t="n">
-        <v>0.2440562130973088</v>
+        <v>0.2440562130973092</v>
       </c>
       <c r="D98" t="n">
-        <v>0.4989555325129462</v>
+        <v>0.4989555325129455</v>
       </c>
     </row>
     <row r="99">
@@ -14620,13 +14667,13 @@
         <v>-2.5</v>
       </c>
       <c r="B99" t="n">
-        <v>0.2829111169380552</v>
+        <v>0.2829111169380555</v>
       </c>
       <c r="C99" t="n">
-        <v>0.2259084276082692</v>
+        <v>0.2259084276082693</v>
       </c>
       <c r="D99" t="n">
-        <v>0.4989602267962243</v>
+        <v>0.498960226796224</v>
       </c>
     </row>
     <row r="100">
@@ -14634,13 +14681,13 @@
         <v>-1.5</v>
       </c>
       <c r="B100" t="n">
-        <v>0.2421545089004232</v>
+        <v>0.2421545089004233</v>
       </c>
       <c r="C100" t="n">
-        <v>0.1663499040174925</v>
+        <v>0.1663499040174926</v>
       </c>
       <c r="D100" t="n">
-        <v>0.4989633527159359</v>
+        <v>0.4989633527159362</v>
       </c>
     </row>
     <row r="101">
@@ -14654,7 +14701,7 @@
         <v>0</v>
       </c>
       <c r="D101" t="n">
-        <v>0.4989649145965428</v>
+        <v>0.4989649145965421</v>
       </c>
     </row>
     <row r="102">
@@ -14668,7 +14715,7 @@
         <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>0.4989649145965428</v>
+        <v>0.4989649145965421</v>
       </c>
     </row>
     <row r="103">
@@ -14676,13 +14723,13 @@
         <v>1.5</v>
       </c>
       <c r="B103" t="n">
-        <v>0.2421545089004232</v>
+        <v>0.2421545089004233</v>
       </c>
       <c r="C103" t="n">
-        <v>0.1663499040174925</v>
+        <v>0.1663499040174926</v>
       </c>
       <c r="D103" t="n">
-        <v>0.4989633527159359</v>
+        <v>0.4989633527159362</v>
       </c>
     </row>
     <row r="104">
@@ -14690,13 +14737,13 @@
         <v>2.5</v>
       </c>
       <c r="B104" t="n">
-        <v>0.2829111169380552</v>
+        <v>0.2829111169380555</v>
       </c>
       <c r="C104" t="n">
-        <v>0.2259084276082692</v>
+        <v>0.2259084276082693</v>
       </c>
       <c r="D104" t="n">
-        <v>0.4989602267962243</v>
+        <v>0.498960226796224</v>
       </c>
     </row>
     <row r="105">
@@ -14704,13 +14751,13 @@
         <v>3.5</v>
       </c>
       <c r="B105" t="n">
-        <v>0.300112390596965</v>
+        <v>0.3001123905969652</v>
       </c>
       <c r="C105" t="n">
-        <v>0.2440562130973088</v>
+        <v>0.2440562130973092</v>
       </c>
       <c r="D105" t="n">
-        <v>0.4989555325129462</v>
+        <v>0.4989555325129455</v>
       </c>
     </row>
     <row r="106">
@@ -14718,13 +14765,13 @@
         <v>4.5</v>
       </c>
       <c r="B106" t="n">
-        <v>0.3352972603430681</v>
+        <v>0.3352972603430684</v>
       </c>
       <c r="C106" t="n">
-        <v>0.2840653476254301</v>
+        <v>0.2840653476254295</v>
       </c>
       <c r="D106" t="n">
-        <v>0.4989492633607075</v>
+        <v>0.4989492633607073</v>
       </c>
     </row>
     <row r="107">
@@ -14732,13 +14779,13 @@
         <v>5.5</v>
       </c>
       <c r="B107" t="n">
-        <v>0.3877315662205335</v>
+        <v>0.3877315662205336</v>
       </c>
       <c r="C107" t="n">
         <v>0.3342570787069619</v>
       </c>
       <c r="D107" t="n">
-        <v>0.4989414106306054</v>
+        <v>0.4989414106306061</v>
       </c>
     </row>
     <row r="108">
@@ -14746,13 +14793,13 @@
         <v>6.5</v>
       </c>
       <c r="B108" t="n">
-        <v>0.4041074485698596</v>
+        <v>0.40410744856986</v>
       </c>
       <c r="C108" t="n">
         <v>0.3682076421570132</v>
       </c>
       <c r="D108" t="n">
-        <v>0.498931963379897</v>
+        <v>0.4989319633798968</v>
       </c>
     </row>
     <row r="109">
@@ -14760,13 +14807,13 @@
         <v>7.5</v>
       </c>
       <c r="B109" t="n">
-        <v>0.4389426994509298</v>
+        <v>0.43894269945093</v>
       </c>
       <c r="C109" t="n">
-        <v>0.38792404962975</v>
+        <v>0.3879240496297497</v>
       </c>
       <c r="D109" t="n">
-        <v>0.4989209083937158</v>
+        <v>0.4989209083937156</v>
       </c>
     </row>
     <row r="110">
@@ -14774,13 +14821,13 @@
         <v>8.5</v>
       </c>
       <c r="B110" t="n">
-        <v>0.4820740942211141</v>
+        <v>0.4820740942211145</v>
       </c>
       <c r="C110" t="n">
         <v>0.4269853796058833</v>
       </c>
       <c r="D110" t="n">
-        <v>0.498908230138588</v>
+        <v>0.4989082301385873</v>
       </c>
     </row>
     <row r="111">
@@ -14788,13 +14835,13 @@
         <v>9.5</v>
       </c>
       <c r="B111" t="n">
-        <v>0.4999181578253317</v>
+        <v>0.4999181578253318</v>
       </c>
       <c r="C111" t="n">
-        <v>0.4653872301930296</v>
+        <v>0.4653872301930295</v>
       </c>
       <c r="D111" t="n">
-        <v>0.4988939107074428</v>
+        <v>0.4988939107074422</v>
       </c>
     </row>
     <row r="112">
@@ -14802,13 +14849,13 @@
         <v>10.5</v>
       </c>
       <c r="B112" t="n">
-        <v>0.5303544982557074</v>
+        <v>0.530354498255708</v>
       </c>
       <c r="C112" t="n">
-        <v>0.4725330359338211</v>
+        <v>0.472533035933821</v>
       </c>
       <c r="D112" t="n">
-        <v>0.4988779297557414</v>
+        <v>0.4988779297557407</v>
       </c>
     </row>
     <row r="113">
@@ -14816,13 +14863,13 @@
         <v>11.5</v>
       </c>
       <c r="B113" t="n">
-        <v>0.539122105997347</v>
+        <v>0.5391221059973471</v>
       </c>
       <c r="C113" t="n">
-        <v>0.5230233532025188</v>
+        <v>0.523023353202519</v>
       </c>
       <c r="D113" t="n">
-        <v>0.4988602644283019</v>
+        <v>0.4988602644283012</v>
       </c>
     </row>
     <row r="114">
@@ -14830,13 +14877,13 @@
         <v>12.5</v>
       </c>
       <c r="B114" t="n">
-        <v>0.5788870879431407</v>
+        <v>0.5788870879431408</v>
       </c>
       <c r="C114" t="n">
-        <v>0.5325837617871744</v>
+        <v>0.5325837617871743</v>
       </c>
       <c r="D114" t="n">
-        <v>0.4988408892763265</v>
+        <v>0.4988408892763267</v>
       </c>
     </row>
     <row r="115">
@@ -14844,13 +14891,13 @@
         <v>13.5</v>
       </c>
       <c r="B115" t="n">
-        <v>0.6011421029666544</v>
+        <v>0.6011421029666546</v>
       </c>
       <c r="C115" t="n">
-        <v>0.5670821387773938</v>
+        <v>0.5670821387773937</v>
       </c>
       <c r="D115" t="n">
-        <v>0.4988197761640505</v>
+        <v>0.4988197761640507</v>
       </c>
     </row>
     <row r="116">
@@ -14858,13 +14905,13 @@
         <v>14.5</v>
       </c>
       <c r="B116" t="n">
-        <v>0.6209617681089237</v>
+        <v>0.6209617681089239</v>
       </c>
       <c r="C116" t="n">
-        <v>0.5921305698265923</v>
+        <v>0.5921305698265928</v>
       </c>
       <c r="D116" t="n">
-        <v>0.4987968941643666</v>
+        <v>0.4987968941643673</v>
       </c>
     </row>
     <row r="117">
@@ -14872,13 +14919,13 @@
         <v>15.5</v>
       </c>
       <c r="B117" t="n">
-        <v>0.6469516045484214</v>
+        <v>0.6469516045484219</v>
       </c>
       <c r="C117" t="n">
-        <v>0.6133578052689883</v>
+        <v>0.6133578052689885</v>
       </c>
       <c r="D117" t="n">
-        <v>0.4987722094426909</v>
+        <v>0.4987722094426906</v>
       </c>
     </row>
     <row r="118">
@@ -14886,13 +14933,13 @@
         <v>16.5</v>
       </c>
       <c r="B118" t="n">
-        <v>0.6669176724807067</v>
+        <v>0.6669176724807072</v>
       </c>
       <c r="C118" t="n">
-        <v>0.6332829617875403</v>
+        <v>0.6332829617875398</v>
       </c>
       <c r="D118" t="n">
-        <v>0.4987456851282283</v>
+        <v>0.4987456851282294</v>
       </c>
     </row>
     <row r="119">
@@ -14900,13 +14947,13 @@
         <v>17.5</v>
       </c>
       <c r="B119" t="n">
-        <v>0.6404980446626786</v>
+        <v>0.6404980446626785</v>
       </c>
       <c r="C119" t="n">
-        <v>0.6101167302671517</v>
+        <v>0.6101167302671512</v>
       </c>
       <c r="D119" t="n">
-        <v>0.4987172811717101</v>
+        <v>0.4987172811717099</v>
       </c>
     </row>
     <row r="120">
@@ -14914,13 +14961,13 @@
         <v>18.5</v>
       </c>
       <c r="B120" t="n">
-        <v>0.671066575295569</v>
+        <v>0.6710665752955695</v>
       </c>
       <c r="C120" t="n">
-        <v>0.6467881970659735</v>
+        <v>0.6467881970659737</v>
       </c>
       <c r="D120" t="n">
-        <v>0.4986869541885289</v>
+        <v>0.4986869541885287</v>
       </c>
     </row>
     <row r="121">
@@ -14928,13 +14975,13 @@
         <v>19.5</v>
       </c>
       <c r="B121" t="n">
-        <v>0.6769639820830026</v>
+        <v>0.6769639820830036</v>
       </c>
       <c r="C121" t="n">
-        <v>0.6608455717034396</v>
+        <v>0.66084557170344</v>
       </c>
       <c r="D121" t="n">
-        <v>0.4986546572861053</v>
+        <v>0.4986546572861046</v>
       </c>
     </row>
     <row r="122">
@@ -14942,13 +14989,13 @@
         <v>20.5</v>
       </c>
       <c r="B122" t="n">
-        <v>0.6813932420874094</v>
+        <v>0.6813932420874093</v>
       </c>
       <c r="C122" t="n">
-        <v>0.6598358656296602</v>
+        <v>0.6598358656296595</v>
       </c>
       <c r="D122" t="n">
-        <v>0.4986203398741444</v>
+        <v>0.4986203398741442</v>
       </c>
     </row>
     <row r="123">
@@ -14956,13 +15003,13 @@
         <v>21.5</v>
       </c>
       <c r="B123" t="n">
-        <v>0.7097767783035674</v>
+        <v>0.7097767783035679</v>
       </c>
       <c r="C123" t="n">
-        <v>0.6805365234859008</v>
+        <v>0.680536523485901</v>
       </c>
       <c r="D123" t="n">
-        <v>0.4985839474562871</v>
+        <v>0.4985839474562869</v>
       </c>
     </row>
     <row r="124">
@@ -14970,13 +15017,13 @@
         <v>22.5</v>
       </c>
       <c r="B124" t="n">
-        <v>0.7003159604390922</v>
+        <v>0.7003159604390918</v>
       </c>
       <c r="C124" t="n">
-        <v>0.6999179633507362</v>
+        <v>0.6999179633507361</v>
       </c>
       <c r="D124" t="n">
-        <v>0.4985454214014907</v>
+        <v>0.4985454214014905</v>
       </c>
     </row>
     <row r="125">
@@ -14984,13 +15031,13 @@
         <v>23.5</v>
       </c>
       <c r="B125" t="n">
-        <v>0.6942382422069006</v>
+        <v>0.6942382422069008</v>
       </c>
       <c r="C125" t="n">
-        <v>0.6979243713813409</v>
+        <v>0.6979243713813407</v>
       </c>
       <c r="D125" t="n">
-        <v>0.4985046986932534</v>
+        <v>0.4985046986932536</v>
       </c>
     </row>
     <row r="126">
@@ -14998,13 +15045,13 @@
         <v>24.5</v>
       </c>
       <c r="B126" t="n">
-        <v>0.7333517317115432</v>
+        <v>0.7333517317115434</v>
       </c>
       <c r="C126" t="n">
-        <v>0.7264060933968987</v>
+        <v>0.7264060933968978</v>
       </c>
       <c r="D126" t="n">
-        <v>0.4984617116545876</v>
+        <v>0.498461711654587</v>
       </c>
     </row>
     <row r="127">
@@ -15012,13 +15059,13 @@
         <v>25.5</v>
       </c>
       <c r="B127" t="n">
-        <v>0.7453626901331355</v>
+        <v>0.7453626901331359</v>
       </c>
       <c r="C127" t="n">
-        <v>0.7717598754606786</v>
+        <v>0.7717598754606784</v>
       </c>
       <c r="D127" t="n">
-        <v>0.4984163876463492</v>
+        <v>0.4984163876463485</v>
       </c>
     </row>
     <row r="128">
@@ -15026,13 +15073,13 @@
         <v>26.5</v>
       </c>
       <c r="B128" t="n">
-        <v>0.7595058745635348</v>
+        <v>0.7595058745635345</v>
       </c>
       <c r="C128" t="n">
-        <v>0.7595896469084757</v>
+        <v>0.7595896469084759</v>
       </c>
       <c r="D128" t="n">
-        <v>0.4983686487363029</v>
+        <v>0.4983686487363018</v>
       </c>
     </row>
     <row r="129">
@@ -15043,10 +15090,10 @@
         <v>0.7738232236139158</v>
       </c>
       <c r="C129" t="n">
-        <v>0.7700672377093174</v>
+        <v>0.7700672377093175</v>
       </c>
       <c r="D129" t="n">
-        <v>0.4983184113358945</v>
+        <v>0.4983184113358947</v>
       </c>
     </row>
     <row r="130">
@@ -15054,13 +15101,13 @@
         <v>28.5</v>
       </c>
       <c r="B130" t="n">
-        <v>0.7848787755905255</v>
+        <v>0.784878775590526</v>
       </c>
       <c r="C130" t="n">
-        <v>0.7822384288115791</v>
+        <v>0.7822384288115796</v>
       </c>
       <c r="D130" t="n">
-        <v>0.4982655858013817</v>
+        <v>0.4982655858013811</v>
       </c>
     </row>
     <row r="131">
@@ -15068,13 +15115,13 @@
         <v>29.5</v>
       </c>
       <c r="B131" t="n">
-        <v>0.754333178138484</v>
+        <v>0.7543331781384839</v>
       </c>
       <c r="C131" t="n">
-        <v>0.7798271559346585</v>
+        <v>0.7798271559346582</v>
       </c>
       <c r="D131" t="n">
-        <v>0.498210075995503</v>
+        <v>0.4982100759955033</v>
       </c>
     </row>
     <row r="132">
@@ -15082,13 +15129,13 @@
         <v>30.5</v>
       </c>
       <c r="B132" t="n">
-        <v>0.7510838934016182</v>
+        <v>0.7510838934016184</v>
       </c>
       <c r="C132" t="n">
-        <v>0.7801299757621555</v>
+        <v>0.7801299757621549</v>
       </c>
       <c r="D132" t="n">
-        <v>0.4981517788054157</v>
+        <v>0.4981517788054154</v>
       </c>
     </row>
     <row r="133">
@@ -15099,10 +15146,10 @@
         <v>0.7621490712918519</v>
       </c>
       <c r="C133" t="n">
-        <v>0.7743819592484078</v>
+        <v>0.7743819592484076</v>
       </c>
       <c r="D133" t="n">
-        <v>0.4980905836120113</v>
+        <v>0.4980905836120115</v>
       </c>
     </row>
     <row r="134">
@@ -15110,13 +15157,13 @@
         <v>32.5</v>
       </c>
       <c r="B134" t="n">
-        <v>0.7658216424068954</v>
+        <v>0.7658216424068957</v>
       </c>
       <c r="C134" t="n">
-        <v>0.762833644079726</v>
+        <v>0.7628336440797258</v>
       </c>
       <c r="D134" t="n">
-        <v>0.4980263717051334</v>
+        <v>0.4980263717051331</v>
       </c>
     </row>
     <row r="135">
@@ -15124,13 +15171,13 @@
         <v>33.5</v>
       </c>
       <c r="B135" t="n">
-        <v>0.7850969335610457</v>
+        <v>0.7850969335610462</v>
       </c>
       <c r="C135" t="n">
-        <v>0.7966176111302646</v>
+        <v>0.7966176111302644</v>
       </c>
       <c r="D135" t="n">
-        <v>0.4979590156384209</v>
+        <v>0.4979590156384207</v>
       </c>
     </row>
     <row r="136">
@@ -15138,13 +15185,13 @@
         <v>34.5</v>
       </c>
       <c r="B136" t="n">
-        <v>0.7786175759937868</v>
+        <v>0.778617575993787</v>
       </c>
       <c r="C136" t="n">
-        <v>0.7944551418583022</v>
+        <v>0.7944551418583017</v>
       </c>
       <c r="D136" t="n">
-        <v>0.4978883785166947</v>
+        <v>0.497888378516694</v>
       </c>
     </row>
     <row r="137">
@@ -15152,13 +15199,13 @@
         <v>35.5</v>
       </c>
       <c r="B137" t="n">
-        <v>0.7475877850546789</v>
+        <v>0.7475877850546786</v>
       </c>
       <c r="C137" t="n">
-        <v>0.7930276421197473</v>
+        <v>0.7930276421197467</v>
       </c>
       <c r="D137" t="n">
-        <v>0.4978143132077587</v>
+        <v>0.497814313207758</v>
       </c>
     </row>
     <row r="138">
@@ -15166,13 +15213,13 @@
         <v>36.5</v>
       </c>
       <c r="B138" t="n">
-        <v>0.7524199679378973</v>
+        <v>0.7524199679378979</v>
       </c>
       <c r="C138" t="n">
-        <v>0.7747048381020563</v>
+        <v>0.7747048381020564</v>
       </c>
       <c r="D138" t="n">
-        <v>0.4977366614693945</v>
+        <v>0.4977366614693943</v>
       </c>
     </row>
     <row r="139">
@@ -15180,13 +15227,13 @@
         <v>37.5</v>
       </c>
       <c r="B139" t="n">
-        <v>0.7920464134216572</v>
+        <v>0.7920464134216577</v>
       </c>
       <c r="C139" t="n">
-        <v>0.7711934302937643</v>
+        <v>0.7711934302937647</v>
       </c>
       <c r="D139" t="n">
-        <v>0.4976552529809558</v>
+        <v>0.497655252980956</v>
       </c>
     </row>
     <row r="140">
@@ -15194,13 +15241,13 @@
         <v>38.5</v>
       </c>
       <c r="B140" t="n">
-        <v>0.7536978025320183</v>
+        <v>0.7536978025320188</v>
       </c>
       <c r="C140" t="n">
-        <v>0.7751001179241852</v>
+        <v>0.7751001179241843</v>
       </c>
       <c r="D140" t="n">
-        <v>0.4975699042674191</v>
+        <v>0.4975699042674197</v>
       </c>
     </row>
     <row r="141">
@@ -15208,13 +15255,13 @@
         <v>39.5</v>
       </c>
       <c r="B141" t="n">
-        <v>0.720475589674085</v>
+        <v>0.7204755896740852</v>
       </c>
       <c r="C141" t="n">
-        <v>0.8117217715841862</v>
+        <v>0.811721771584186</v>
       </c>
       <c r="D141" t="n">
-        <v>0.4974804175019663</v>
+        <v>0.4974804175019656</v>
       </c>
     </row>
     <row r="142">
@@ -15222,13 +15269,13 @@
         <v>40.5</v>
       </c>
       <c r="B142" t="n">
-        <v>0.6926928773884129</v>
+        <v>0.6926928773884131</v>
       </c>
       <c r="C142" t="n">
-        <v>0.7754443003335992</v>
+        <v>0.775444300333599</v>
       </c>
       <c r="D142" t="n">
-        <v>0.4973865791710019</v>
+        <v>0.4973865791710017</v>
       </c>
     </row>
     <row r="143">
@@ -15236,13 +15283,13 @@
         <v>41.5</v>
       </c>
       <c r="B143" t="n">
-        <v>0.6756810914760258</v>
+        <v>0.675681091476026</v>
       </c>
       <c r="C143" t="n">
-        <v>0.7475540536762612</v>
+        <v>0.7475540536762606</v>
       </c>
       <c r="D143" t="n">
-        <v>0.4972881585830732</v>
+        <v>0.497288158583073</v>
       </c>
     </row>
     <row r="144">
@@ -15250,13 +15297,13 @@
         <v>42.5</v>
       </c>
       <c r="B144" t="n">
-        <v>0.6656779753720748</v>
+        <v>0.6656779753720753</v>
       </c>
       <c r="C144" t="n">
-        <v>0.7346912850045731</v>
+        <v>0.734691285004573</v>
       </c>
       <c r="D144" t="n">
-        <v>0.4971849062001671</v>
+        <v>0.4971849062001669</v>
       </c>
     </row>
     <row r="145">
@@ -15264,13 +15311,13 @@
         <v>43.5</v>
       </c>
       <c r="B145" t="n">
-        <v>0.6614806547034983</v>
+        <v>0.6614806547034987</v>
       </c>
       <c r="C145" t="n">
-        <v>0.7007304608014034</v>
+        <v>0.700730460801403</v>
       </c>
       <c r="D145" t="n">
-        <v>0.497076551766442</v>
+        <v>0.4970765517664418</v>
       </c>
     </row>
     <row r="146">
@@ -15278,13 +15325,13 @@
         <v>44.5</v>
       </c>
       <c r="B146" t="n">
-        <v>0.6579346460701211</v>
+        <v>0.6579346460701213</v>
       </c>
       <c r="C146" t="n">
-        <v>0.6855482572812029</v>
+        <v>0.6855482572812028</v>
       </c>
       <c r="D146" t="n">
-        <v>0.4969628022053188</v>
+        <v>0.4969628022053186</v>
       </c>
     </row>
     <row r="147">
@@ -15292,13 +15339,13 @@
         <v>45.5</v>
       </c>
       <c r="B147" t="n">
-        <v>0.65703046610319</v>
+        <v>0.6570304661031902</v>
       </c>
       <c r="C147" t="n">
-        <v>0.6891287255111701</v>
+        <v>0.68912872551117</v>
       </c>
       <c r="D147" t="n">
-        <v>0.4968433392509789</v>
+        <v>0.4968433392509787</v>
       </c>
     </row>
     <row r="148">
@@ -15306,13 +15353,13 @@
         <v>46.5</v>
       </c>
       <c r="B148" t="n">
-        <v>0.6523653457907461</v>
+        <v>0.6523653457907458</v>
       </c>
       <c r="C148" t="n">
-        <v>0.6938881629172772</v>
+        <v>0.693888162917277</v>
       </c>
       <c r="D148" t="n">
-        <v>0.4967178167744916</v>
+        <v>0.4967178167744914</v>
       </c>
     </row>
     <row r="149">
@@ -15320,13 +15367,13 @@
         <v>47.5</v>
       </c>
       <c r="B149" t="n">
-        <v>0.6560576920298822</v>
+        <v>0.6560576920298824</v>
       </c>
       <c r="C149" t="n">
-        <v>0.6759809314377453</v>
+        <v>0.6759809314377454</v>
       </c>
       <c r="D149" t="n">
-        <v>0.4965858577578205</v>
+        <v>0.4965858577578208</v>
       </c>
     </row>
     <row r="150">
@@ -15334,13 +15381,13 @@
         <v>48.5</v>
       </c>
       <c r="B150" t="n">
-        <v>0.6422987617800502</v>
+        <v>0.6422987617800497</v>
       </c>
       <c r="C150" t="n">
-        <v>0.6828565450664376</v>
+        <v>0.6828565450664378</v>
       </c>
       <c r="D150" t="n">
-        <v>0.496447050860586</v>
+        <v>0.4964470508605858</v>
       </c>
     </row>
     <row r="151">
@@ -15348,13 +15395,13 @@
         <v>49.5</v>
       </c>
       <c r="B151" t="n">
-        <v>0.6296245049056135</v>
+        <v>0.6296245049056137</v>
       </c>
       <c r="C151" t="n">
-        <v>0.7021565699010888</v>
+        <v>0.7021565699010887</v>
       </c>
       <c r="D151" t="n">
-        <v>0.496300946514333</v>
+        <v>0.4963009465143333</v>
       </c>
     </row>
     <row r="152">
@@ -15362,13 +15409,13 @@
         <v>50.5</v>
       </c>
       <c r="B152" t="n">
-        <v>0.629700875046741</v>
+        <v>0.6297008750467409</v>
       </c>
       <c r="C152" t="n">
-        <v>0.6784468564926708</v>
+        <v>0.6784468564926709</v>
       </c>
       <c r="D152" t="n">
-        <v>0.4961470524668356</v>
+        <v>0.4961470524668354</v>
       </c>
     </row>
     <row r="153">
@@ -15376,13 +15423,13 @@
         <v>51.5</v>
       </c>
       <c r="B153" t="n">
-        <v>0.6482710607618596</v>
+        <v>0.6482710607618598</v>
       </c>
       <c r="C153" t="n">
-        <v>0.6444745327159636</v>
+        <v>0.6444745327159631</v>
       </c>
       <c r="D153" t="n">
-        <v>0.4959848286840581</v>
+        <v>0.4959848286840583</v>
       </c>
     </row>
     <row r="154">
@@ -15390,13 +15437,13 @@
         <v>52.5</v>
       </c>
       <c r="B154" t="n">
-        <v>0.6621240246579133</v>
+        <v>0.6621240246579135</v>
       </c>
       <c r="C154" t="n">
-        <v>0.6608141905780918</v>
+        <v>0.660814190578092</v>
       </c>
       <c r="D154" t="n">
-        <v>0.495813681499212</v>
+        <v>0.4958136814992118</v>
       </c>
     </row>
     <row r="155">
@@ -15404,13 +15451,13 @@
         <v>53.5</v>
       </c>
       <c r="B155" t="n">
-        <v>0.6075886268367905</v>
+        <v>0.6075886268367907</v>
       </c>
       <c r="C155" t="n">
-        <v>0.6417492754696281</v>
+        <v>0.6417492754696279</v>
       </c>
       <c r="D155" t="n">
-        <v>0.4956329568760179</v>
+        <v>0.4956329568760177</v>
       </c>
     </row>
     <row r="156">
@@ -15418,13 +15465,13 @@
         <v>54.5</v>
       </c>
       <c r="B156" t="n">
-        <v>0.6145222782996753</v>
+        <v>0.6145222782996752</v>
       </c>
       <c r="C156" t="n">
-        <v>0.6955921174697973</v>
+        <v>0.6955921174697978</v>
       </c>
       <c r="D156" t="n">
-        <v>0.4954419326257448</v>
+        <v>0.4954419326257442</v>
       </c>
     </row>
     <row r="157">
@@ -15432,13 +15479,13 @@
         <v>55.5</v>
       </c>
       <c r="B157" t="n">
-        <v>0.626859395629082</v>
+        <v>0.6268593956290824</v>
       </c>
       <c r="C157" t="n">
-        <v>0.6140979057477214</v>
+        <v>0.6140979057477209</v>
       </c>
       <c r="D157" t="n">
-        <v>0.4952398093834697</v>
+        <v>0.4952398093834686</v>
       </c>
     </row>
     <row r="158">
@@ -15446,13 +15493,13 @@
         <v>56.5</v>
       </c>
       <c r="B158" t="n">
-        <v>0.6269512787918737</v>
+        <v>0.6269512787918736</v>
       </c>
       <c r="C158" t="n">
-        <v>0.6219176561838072</v>
+        <v>0.6219176561838073</v>
       </c>
       <c r="D158" t="n">
-        <v>0.4950257001064756</v>
+        <v>0.4950257001064754</v>
       </c>
     </row>
     <row r="159">
@@ -15460,13 +15507,13 @@
         <v>57.5</v>
       </c>
       <c r="B159" t="n">
-        <v>0.6043557745641925</v>
+        <v>0.6043557745641932</v>
       </c>
       <c r="C159" t="n">
-        <v>0.6196484289744897</v>
+        <v>0.6196484289744902</v>
       </c>
       <c r="D159" t="n">
-        <v>0.4947986178044071</v>
+        <v>0.4947986178044065</v>
       </c>
     </row>
     <row r="160">
@@ -15474,13 +15521,13 @@
         <v>58.5</v>
       </c>
       <c r="B160" t="n">
-        <v>0.6099279444003927</v>
+        <v>0.6099279444003929</v>
       </c>
       <c r="C160" t="n">
-        <v>0.6414397726211378</v>
+        <v>0.641439772621138</v>
       </c>
       <c r="D160" t="n">
-        <v>0.4945574611436202</v>
+        <v>0.4945574611436195</v>
       </c>
     </row>
     <row r="161">
@@ -15488,13 +15535,13 @@
         <v>59.5</v>
       </c>
       <c r="B161" t="n">
-        <v>0.5994710980975342</v>
+        <v>0.5994710980975344</v>
       </c>
       <c r="C161" t="n">
-        <v>0.6282379761625425</v>
+        <v>0.6282379761625431</v>
       </c>
       <c r="D161" t="n">
-        <v>0.4943009974829747</v>
+        <v>0.494300997482974</v>
       </c>
     </row>
     <row r="162">
@@ -15502,13 +15549,13 @@
         <v>60.5</v>
       </c>
       <c r="B162" t="n">
-        <v>0.6079992034749827</v>
+        <v>0.6079992034749826</v>
       </c>
       <c r="C162" t="n">
-        <v>0.6152754383834582</v>
+        <v>0.615275438383458</v>
       </c>
       <c r="D162" t="n">
-        <v>0.4940278427895055</v>
+        <v>0.4940278427895053</v>
       </c>
     </row>
     <row r="163">
@@ -15516,13 +15563,13 @@
         <v>61.5</v>
       </c>
       <c r="B163" t="n">
-        <v>0.6282769128884991</v>
+        <v>0.6282769128884992</v>
       </c>
       <c r="C163" t="n">
-        <v>0.6205640652875102</v>
+        <v>0.62056406528751</v>
       </c>
       <c r="D163" t="n">
-        <v>0.493736437742581</v>
+        <v>0.4937364377425812</v>
       </c>
     </row>
     <row r="164">
@@ -15530,13 +15577,13 @@
         <v>62.5</v>
       </c>
       <c r="B164" t="n">
-        <v>0.6133028294805949</v>
+        <v>0.6133028294805953</v>
       </c>
       <c r="C164" t="n">
-        <v>0.6030626920559258</v>
+        <v>0.6030626920559257</v>
       </c>
       <c r="D164" t="n">
-        <v>0.4934250191540233</v>
+        <v>0.4934250191540226</v>
       </c>
     </row>
     <row r="165">
@@ -15544,13 +15591,13 @@
         <v>63.5</v>
       </c>
       <c r="B165" t="n">
-        <v>0.6080531387907387</v>
+        <v>0.608053138790739</v>
       </c>
       <c r="C165" t="n">
-        <v>0.6023853488338297</v>
+        <v>0.6023853488338292</v>
       </c>
       <c r="D165" t="n">
-        <v>0.4930915855952366</v>
+        <v>0.4930915855952364</v>
       </c>
     </row>
     <row r="166">
@@ -15558,13 +15605,13 @@
         <v>64.5</v>
       </c>
       <c r="B166" t="n">
-        <v>0.6515817250481675</v>
+        <v>0.6515817250481679</v>
       </c>
       <c r="C166" t="n">
-        <v>0.612716109480149</v>
+        <v>0.6127161094801492</v>
       </c>
       <c r="D166" t="n">
-        <v>0.4927338558112788</v>
+        <v>0.4927338558112785</v>
       </c>
     </row>
     <row r="167">
@@ -15572,13 +15619,13 @@
         <v>65.5</v>
       </c>
       <c r="B167" t="n">
-        <v>0.6343327075976388</v>
+        <v>0.6343327075976387</v>
       </c>
       <c r="C167" t="n">
-        <v>0.5956839979554051</v>
+        <v>0.5956839979554049</v>
       </c>
       <c r="D167" t="n">
-        <v>0.4923492180885909</v>
+        <v>0.4923492180885911</v>
       </c>
     </row>
     <row r="168">
@@ -15586,13 +15633,13 @@
         <v>66.5</v>
       </c>
       <c r="B168" t="n">
-        <v>0.6704217975309409</v>
+        <v>0.6704217975309414</v>
       </c>
       <c r="C168" t="n">
-        <v>0.6100115711576957</v>
+        <v>0.6100115711576956</v>
       </c>
       <c r="D168" t="n">
-        <v>0.4919346681893128</v>
+        <v>0.4919346681893125</v>
       </c>
     </row>
     <row r="169">
@@ -15600,13 +15647,13 @@
         <v>67.5</v>
       </c>
       <c r="B169" t="n">
-        <v>0.6854921487171532</v>
+        <v>0.6854921487171537</v>
       </c>
       <c r="C169" t="n">
-        <v>0.6282920299046594</v>
+        <v>0.6282920299046593</v>
       </c>
       <c r="D169" t="n">
-        <v>0.4914867327150998</v>
+        <v>0.4914867327150996</v>
       </c>
     </row>
     <row r="170">
@@ -15617,10 +15664,10 @@
         <v>0.6968852396108124</v>
       </c>
       <c r="C170" t="n">
-        <v>0.6532069208884197</v>
+        <v>0.6532069208884193</v>
       </c>
       <c r="D170" t="n">
-        <v>0.4910013737367041</v>
+        <v>0.491001373736703</v>
       </c>
     </row>
     <row r="171">
@@ -15628,13 +15675,13 @@
         <v>69.5</v>
       </c>
       <c r="B171" t="n">
-        <v>0.7403937167767312</v>
+        <v>0.7403937167767317</v>
       </c>
       <c r="C171" t="n">
-        <v>0.6984860950493469</v>
+        <v>0.6984860950493468</v>
       </c>
       <c r="D171" t="n">
-        <v>0.4904738691034787</v>
+        <v>0.4904738691034785</v>
       </c>
     </row>
     <row r="172">
@@ -15642,13 +15689,13 @@
         <v>70.5</v>
       </c>
       <c r="B172" t="n">
-        <v>0.7359459575879775</v>
+        <v>0.7359459575879777</v>
       </c>
       <c r="C172" t="n">
-        <v>0.663419677775356</v>
+        <v>0.6634196777753558</v>
       </c>
       <c r="D172" t="n">
-        <v>0.4898986608521688</v>
+        <v>0.4898986608521677</v>
       </c>
     </row>
     <row r="173">
@@ -15656,13 +15703,13 @@
         <v>71.5</v>
       </c>
       <c r="B173" t="n">
-        <v>0.7551819610901543</v>
+        <v>0.7551819610901546</v>
       </c>
       <c r="C173" t="n">
-        <v>0.6651581063795067</v>
+        <v>0.6651581063795066</v>
       </c>
       <c r="D173" t="n">
-        <v>0.4892691612972991</v>
+        <v>0.4892691612972989</v>
       </c>
     </row>
     <row r="174">
@@ -15670,13 +15717,13 @@
         <v>72.5</v>
       </c>
       <c r="B174" t="n">
-        <v>0.7525718692087209</v>
+        <v>0.7525718692087211</v>
       </c>
       <c r="C174" t="n">
-        <v>0.6846515295886507</v>
+        <v>0.6846515295886506</v>
       </c>
       <c r="D174" t="n">
-        <v>0.4885775022900861</v>
+        <v>0.4885775022900855</v>
       </c>
     </row>
     <row r="175">
@@ -15684,13 +15731,13 @@
         <v>73.5</v>
       </c>
       <c r="B175" t="n">
-        <v>0.7614903717084363</v>
+        <v>0.7614903717084365</v>
       </c>
       <c r="C175" t="n">
-        <v>0.7317342294921181</v>
+        <v>0.7317342294921179</v>
       </c>
       <c r="D175" t="n">
-        <v>0.4878142071232827</v>
+        <v>0.4878142071232824</v>
       </c>
     </row>
     <row r="176">
@@ -15698,13 +15745,13 @@
         <v>74.5</v>
       </c>
       <c r="B176" t="n">
-        <v>0.7944189533381556</v>
+        <v>0.7944189533381555</v>
       </c>
       <c r="C176" t="n">
-        <v>0.7574846670879898</v>
+        <v>0.7574846670879899</v>
       </c>
       <c r="D176" t="n">
-        <v>0.4869677555819383</v>
+        <v>0.4869677555819381</v>
       </c>
     </row>
     <row r="177">
@@ -15712,13 +15759,13 @@
         <v>75.5</v>
       </c>
       <c r="B177" t="n">
-        <v>0.8226512579916015</v>
+        <v>0.8226512579916018</v>
       </c>
       <c r="C177" t="n">
-        <v>0.7559103261366089</v>
+        <v>0.755910326136608</v>
       </c>
       <c r="D177" t="n">
-        <v>0.486023998960846</v>
+        <v>0.4860239989608462</v>
       </c>
     </row>
     <row r="178">
@@ -15726,13 +15773,13 @@
         <v>76.5</v>
       </c>
       <c r="B178" t="n">
-        <v>0.8234536853907762</v>
+        <v>0.8234536853907765</v>
       </c>
       <c r="C178" t="n">
-        <v>0.8038133418703667</v>
+        <v>0.8038133418703661</v>
       </c>
       <c r="D178" t="n">
-        <v>0.4849653605638656</v>
+        <v>0.4849653605638654</v>
       </c>
     </row>
     <row r="179">
@@ -15743,10 +15790,10 @@
         <v>0.8427787165576837</v>
       </c>
       <c r="C179" t="n">
-        <v>0.8315160483471457</v>
+        <v>0.8315160483471453</v>
       </c>
       <c r="D179" t="n">
-        <v>0.4837697231935115</v>
+        <v>0.4837697231935117</v>
       </c>
     </row>
     <row r="180">
@@ -15754,13 +15801,13 @@
         <v>78.5</v>
       </c>
       <c r="B180" t="n">
-        <v>0.8588143440805717</v>
+        <v>0.8588143440805713</v>
       </c>
       <c r="C180" t="n">
-        <v>0.8577225764872749</v>
+        <v>0.857722576487274</v>
       </c>
       <c r="D180" t="n">
-        <v>0.4824088493430208</v>
+        <v>0.482408849343021</v>
       </c>
     </row>
     <row r="181">
@@ -15768,13 +15815,13 @@
         <v>79.5</v>
       </c>
       <c r="B181" t="n">
-        <v>0.8590822225198615</v>
+        <v>0.859082222519862</v>
       </c>
       <c r="C181" t="n">
         <v>0.8686954244354625</v>
       </c>
       <c r="D181" t="n">
-        <v>0.4808460853500087</v>
+        <v>0.4808460853500089</v>
       </c>
     </row>
     <row r="182">
@@ -15782,13 +15829,13 @@
         <v>80.5</v>
       </c>
       <c r="B182" t="n">
-        <v>0.9073459952330268</v>
+        <v>0.9073459952330274</v>
       </c>
       <c r="C182" t="n">
-        <v>0.8922182310421599</v>
+        <v>0.8922182310421597</v>
       </c>
       <c r="D182" t="n">
-        <v>0.4790329350508588</v>
+        <v>0.4790329350508589</v>
       </c>
     </row>
     <row r="183">
@@ -15796,13 +15843,13 @@
         <v>81.5</v>
       </c>
       <c r="B183" t="n">
-        <v>0.949005915299686</v>
+        <v>0.9490059152996863</v>
       </c>
       <c r="C183" t="n">
-        <v>0.9203255877950701</v>
+        <v>0.9203255877950698</v>
       </c>
       <c r="D183" t="n">
-        <v>0.4769037854021088</v>
+        <v>0.4769037854021086</v>
       </c>
     </row>
     <row r="184">
@@ -15810,13 +15857,13 @@
         <v>82.5</v>
       </c>
       <c r="B184" t="n">
-        <v>0.9422191298223839</v>
+        <v>0.9422191298223848</v>
       </c>
       <c r="C184" t="n">
-        <v>0.936050289253903</v>
+        <v>0.9360502892539027</v>
       </c>
       <c r="D184" t="n">
-        <v>0.4743674845947118</v>
+        <v>0.4743674845947116</v>
       </c>
     </row>
     <row r="185">
@@ -15824,13 +15871,13 @@
         <v>83.5</v>
       </c>
       <c r="B185" t="n">
-        <v>0.9504237461131312</v>
+        <v>0.950423746113132</v>
       </c>
       <c r="C185" t="n">
-        <v>0.9022084139331087</v>
+        <v>0.9022084139331085</v>
       </c>
       <c r="D185" t="n">
-        <v>0.4712932888281461</v>
+        <v>0.4712932888281459</v>
       </c>
     </row>
     <row r="186">
@@ -15838,13 +15885,13 @@
         <v>84.5</v>
       </c>
       <c r="B186" t="n">
-        <v>0.9348241708469139</v>
+        <v>0.9348241708469145</v>
       </c>
       <c r="C186" t="n">
-        <v>0.9996418421698857</v>
+        <v>0.9996418421698854</v>
       </c>
       <c r="D186" t="n">
-        <v>0.4674861062426789</v>
+        <v>0.4674861062426786</v>
       </c>
     </row>
     <row r="187">
@@ -15852,13 +15899,13 @@
         <v>85.5</v>
       </c>
       <c r="B187" t="n">
-        <v>0.9396782260874059</v>
+        <v>0.9396782260874063</v>
       </c>
       <c r="C187" t="n">
         <v>0.9958274071033653</v>
       </c>
       <c r="D187" t="n">
-        <v>0.4626397873271937</v>
+        <v>0.4626397873271935</v>
       </c>
     </row>
     <row r="188">
@@ -15866,13 +15913,13 @@
         <v>86.5</v>
       </c>
       <c r="B188" t="n">
-        <v>0.9574561212793653</v>
+        <v>0.9574561212793656</v>
       </c>
       <c r="C188" t="n">
-        <v>0.9936465196613629</v>
+        <v>0.9936465196613622</v>
       </c>
       <c r="D188" t="n">
-        <v>0.4562406525897308</v>
+        <v>0.4562406525897311</v>
       </c>
     </row>
     <row r="189">
@@ -15880,13 +15927,13 @@
         <v>87.5</v>
       </c>
       <c r="B189" t="n">
-        <v>0.9526932718290473</v>
+        <v>0.9526932718290475</v>
       </c>
       <c r="C189" t="n">
         <v>1</v>
       </c>
       <c r="D189" t="n">
-        <v>0.4473415281371259</v>
+        <v>0.4473415281371261</v>
       </c>
     </row>
     <row r="190">
@@ -15897,10 +15944,10 @@
         <v>1</v>
       </c>
       <c r="C190" t="n">
-        <v>0.9826620006446274</v>
+        <v>0.9826620006446267</v>
       </c>
       <c r="D190" t="n">
-        <v>0.4339215502290429</v>
+        <v>0.4339215502290431</v>
       </c>
     </row>
     <row r="191">
@@ -15908,13 +15955,13 @@
         <v>89.5</v>
       </c>
       <c r="B191" t="n">
-        <v>0.920034786848233</v>
+        <v>0.9200347868482333</v>
       </c>
       <c r="C191" t="n">
-        <v>0.9576065329048673</v>
+        <v>0.9576065329048666</v>
       </c>
       <c r="D191" t="n">
-        <v>0.4103572060618615</v>
+        <v>0.4103572060618613</v>
       </c>
     </row>
     <row r="192">
@@ -15925,10 +15972,10 @@
         <v>0.9099481169834489</v>
       </c>
       <c r="C192" t="n">
-        <v>0.9701009922984414</v>
+        <v>0.970100992298441</v>
       </c>
       <c r="D192" t="n">
-        <v>0.3446638354971175</v>
+        <v>0.3446638354971177</v>
       </c>
     </row>
     <row r="193">
@@ -15936,13 +15983,13 @@
         <v>91.5</v>
       </c>
       <c r="B193" t="n">
-        <v>0.9181860521551287</v>
+        <v>0.9181860521551291</v>
       </c>
       <c r="C193" t="n">
-        <v>0.9948473801037144</v>
+        <v>0.9948473801037139</v>
       </c>
       <c r="D193" t="n">
-        <v>0.5541061527117704</v>
+        <v>0.5541061527117702</v>
       </c>
     </row>
     <row r="194">
@@ -15953,10 +16000,10 @@
         <v>0.8857752764382696</v>
       </c>
       <c r="C194" t="n">
-        <v>0.9436124218256501</v>
+        <v>0.9436124218256494</v>
       </c>
       <c r="D194" t="n">
-        <v>0.5170396654691453</v>
+        <v>0.517039665469145</v>
       </c>
     </row>
     <row r="195">
@@ -15964,13 +16011,13 @@
         <v>93.5</v>
       </c>
       <c r="B195" t="n">
-        <v>0.9166586588809894</v>
+        <v>0.9166586588809902</v>
       </c>
       <c r="C195" t="n">
-        <v>0.8720846784569759</v>
+        <v>0.8720846784569756</v>
       </c>
       <c r="D195" t="n">
-        <v>0.816583536027413</v>
+        <v>0.8165835360274134</v>
       </c>
     </row>
     <row r="196">
@@ -15981,10 +16028,10 @@
         <v>0.8580910676842974</v>
       </c>
       <c r="C196" t="n">
-        <v>0.8784181899133735</v>
+        <v>0.8784181899133733</v>
       </c>
       <c r="D196" t="n">
-        <v>0.8327479931898826</v>
+        <v>0.832747993189883</v>
       </c>
     </row>
     <row r="197">
@@ -15992,13 +16039,13 @@
         <v>95.5</v>
       </c>
       <c r="B197" t="n">
-        <v>0.8788090083020381</v>
+        <v>0.8788090083020387</v>
       </c>
       <c r="C197" t="n">
-        <v>0.9268316030667308</v>
+        <v>0.9268316030667305</v>
       </c>
       <c r="D197" t="n">
-        <v>0.640454327416757</v>
+        <v>0.6404543274167573</v>
       </c>
     </row>
     <row r="198">
@@ -16006,13 +16053,13 @@
         <v>96.5</v>
       </c>
       <c r="B198" t="n">
-        <v>0.830806726222212</v>
+        <v>0.8308067262222125</v>
       </c>
       <c r="C198" t="n">
-        <v>0.8548773313478353</v>
+        <v>0.8548773313478354</v>
       </c>
       <c r="D198" t="n">
-        <v>0.7346087745699452</v>
+        <v>0.7346087745699451</v>
       </c>
     </row>
     <row r="199">
@@ -16023,7 +16070,7 @@
         <v>0.6589791116939901</v>
       </c>
       <c r="C199" t="n">
-        <v>0.7645900931604129</v>
+        <v>0.7645900931604124</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -16034,13 +16081,13 @@
         <v>98.5</v>
       </c>
       <c r="B200" t="n">
-        <v>0.5701292827038069</v>
+        <v>0.5701292827038071</v>
       </c>
       <c r="C200" t="n">
-        <v>0.5533316101628996</v>
+        <v>0.5533316101628994</v>
       </c>
       <c r="D200" t="n">
-        <v>0.8438845951917385</v>
+        <v>0.8438845951917384</v>
       </c>
     </row>
     <row r="201">
@@ -16072,17 +16119,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>